<commit_message>
Bookmark way of filling the form
</commit_message>
<xml_diff>
--- a/InputTransactionDataHarder.xlsx
+++ b/InputTransactionDataHarder.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\dev\UIpath Ciphix\Ciphix_air_UI\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\dev\UIpath Ciphix\Ciphix_Air\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C3B6292-3020-4A21-9F7F-48C650EC4C1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4975FBC-A5A1-4133-BB6A-F24F0556D061}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38510" yWindow="-930" windowWidth="38620" windowHeight="21100" xr2:uid="{8E712073-4D35-4677-80EE-D80F1EA3F2D9}"/>
+    <workbookView xWindow="28680" yWindow="-1350" windowWidth="38640" windowHeight="21120" xr2:uid="{8E712073-4D35-4677-80EE-D80F1EA3F2D9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="60">
   <si>
     <t>Age</t>
   </si>
@@ -556,7 +556,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63DB6C32-5833-4D0B-AC7B-28C7DFA19D6B}">
-  <dimension ref="A1:K35"/>
+  <dimension ref="A1:K29"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="13.5703125" customWidth="1"/>
@@ -606,1093 +606,895 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C2">
+        <v>84963</v>
+      </c>
+      <c r="D2" t="s">
+        <v>53</v>
+      </c>
+      <c r="E2" t="s">
+        <v>57</v>
+      </c>
+      <c r="F2">
         <v>21</v>
       </c>
-      <c r="B2" t="s">
-        <v>28</v>
-      </c>
-      <c r="C2">
-        <v>30307</v>
-      </c>
-      <c r="D2" t="s">
-        <v>41</v>
-      </c>
-      <c r="E2" t="s">
-        <v>1</v>
-      </c>
-      <c r="F2">
-        <v>24</v>
-      </c>
       <c r="G2" t="s">
-        <v>33</v>
+        <v>54</v>
       </c>
       <c r="H2" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="I2">
-        <v>154</v>
+        <v>56</v>
+      </c>
+      <c r="J2" t="s">
+        <v>48</v>
       </c>
       <c r="K2" t="s">
-        <v>8</v>
+        <v>56</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C3">
-        <v>35454</v>
+        <v>30307</v>
       </c>
       <c r="D3" t="s">
-        <v>14</v>
+        <v>41</v>
       </c>
       <c r="E3" t="s">
-        <v>46</v>
+        <v>1</v>
       </c>
       <c r="F3">
-        <v>55</v>
+        <v>24</v>
       </c>
       <c r="G3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H3" t="s">
-        <v>35</v>
+        <v>47</v>
       </c>
       <c r="I3">
-        <v>60</v>
-      </c>
-      <c r="J3" t="s">
-        <v>48</v>
+        <v>154</v>
       </c>
       <c r="K3" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B4" t="s">
         <v>27</v>
       </c>
       <c r="C4">
-        <v>13703</v>
+        <v>35454</v>
       </c>
       <c r="D4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E4" t="s">
-        <v>16</v>
+        <v>46</v>
       </c>
       <c r="F4">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="G4" t="s">
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="H4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="I4">
-        <v>24</v>
+        <v>60</v>
+      </c>
+      <c r="J4" t="s">
+        <v>48</v>
       </c>
       <c r="K4" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>23</v>
+      </c>
+      <c r="B5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5">
+        <v>13703</v>
+      </c>
+      <c r="D5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E5" t="s">
+        <v>16</v>
+      </c>
+      <c r="F5">
+        <v>44</v>
+      </c>
+      <c r="G5" t="s">
+        <v>49</v>
+      </c>
+      <c r="H5" t="s">
+        <v>36</v>
+      </c>
+      <c r="I5">
         <v>24</v>
       </c>
-      <c r="B5" t="s">
-        <v>30</v>
-      </c>
-      <c r="C5">
-        <v>25633</v>
-      </c>
-      <c r="D5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F5">
-        <v>33</v>
-      </c>
-      <c r="G5" t="s">
-        <v>38</v>
-      </c>
-      <c r="H5" t="s">
-        <v>39</v>
-      </c>
-      <c r="I5">
-        <v>10</v>
-      </c>
       <c r="K5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C6">
-        <v>32961</v>
+        <v>25633</v>
       </c>
       <c r="D6" t="s">
-        <v>43</v>
+        <v>17</v>
       </c>
       <c r="E6" t="s">
-        <v>45</v>
+        <v>18</v>
       </c>
       <c r="F6">
-        <v>21</v>
+        <v>33</v>
       </c>
       <c r="G6" t="s">
-        <v>58</v>
+        <v>38</v>
       </c>
       <c r="H6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="I6">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="K6" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C7">
-        <v>17107</v>
+        <v>32961</v>
       </c>
       <c r="D7" t="s">
-        <v>19</v>
+        <v>43</v>
       </c>
       <c r="E7" t="s">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="F7">
-        <v>44</v>
+        <v>21</v>
       </c>
       <c r="G7" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="H7" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="I7">
-        <v>17</v>
-      </c>
-      <c r="J7" t="s">
-        <v>48</v>
+        <v>5</v>
       </c>
       <c r="K7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>51</v>
+        <v>26</v>
       </c>
       <c r="B8" t="s">
-        <v>52</v>
+        <v>30</v>
       </c>
       <c r="C8">
-        <v>84963</v>
+        <v>17107</v>
       </c>
       <c r="D8" t="s">
-        <v>53</v>
+        <v>19</v>
       </c>
       <c r="E8" t="s">
-        <v>57</v>
+        <v>20</v>
       </c>
       <c r="F8">
-        <v>21</v>
+        <v>44</v>
       </c>
       <c r="G8" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="H8" t="s">
-        <v>55</v>
+        <v>44</v>
       </c>
       <c r="I8">
-        <v>56</v>
+        <v>17</v>
       </c>
       <c r="J8" t="s">
         <v>48</v>
       </c>
       <c r="K8" t="s">
-        <v>56</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>51</v>
+      </c>
+      <c r="B9" t="s">
+        <v>52</v>
+      </c>
+      <c r="C9">
+        <v>84963</v>
+      </c>
+      <c r="D9" t="s">
+        <v>53</v>
+      </c>
+      <c r="E9" t="s">
+        <v>57</v>
+      </c>
+      <c r="F9">
         <v>21</v>
       </c>
-      <c r="B9" t="s">
-        <v>28</v>
-      </c>
-      <c r="C9">
-        <v>30307</v>
-      </c>
-      <c r="D9" t="s">
-        <v>41</v>
-      </c>
-      <c r="E9" t="s">
-        <v>1</v>
-      </c>
-      <c r="F9">
-        <v>24</v>
-      </c>
       <c r="G9" t="s">
-        <v>33</v>
+        <v>54</v>
       </c>
       <c r="H9" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="I9">
-        <v>154</v>
+        <v>56</v>
+      </c>
+      <c r="J9" t="s">
+        <v>48</v>
       </c>
       <c r="K9" t="s">
-        <v>8</v>
+        <v>56</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B10" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C10">
-        <v>35454</v>
+        <v>25641</v>
       </c>
       <c r="D10" t="s">
-        <v>14</v>
+        <v>41</v>
       </c>
       <c r="E10" t="s">
-        <v>46</v>
+        <v>1</v>
       </c>
       <c r="F10">
-        <v>55</v>
+        <v>24</v>
       </c>
       <c r="G10" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H10" t="s">
-        <v>35</v>
+        <v>47</v>
       </c>
       <c r="I10">
-        <v>60</v>
-      </c>
-      <c r="J10" t="s">
-        <v>48</v>
+        <v>154</v>
       </c>
       <c r="K10" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B11" t="s">
         <v>27</v>
       </c>
       <c r="C11">
-        <v>13703</v>
+        <v>78945</v>
       </c>
       <c r="D11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E11" t="s">
-        <v>16</v>
+        <v>46</v>
       </c>
       <c r="F11">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="G11" t="s">
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="H11" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="I11">
-        <v>24</v>
+        <v>60</v>
+      </c>
+      <c r="J11" t="s">
+        <v>48</v>
       </c>
       <c r="K11" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>23</v>
+      </c>
+      <c r="B12" t="s">
+        <v>27</v>
+      </c>
+      <c r="C12">
+        <v>25846</v>
+      </c>
+      <c r="D12" t="s">
+        <v>15</v>
+      </c>
+      <c r="E12" t="s">
+        <v>16</v>
+      </c>
+      <c r="F12">
+        <v>44</v>
+      </c>
+      <c r="G12" t="s">
+        <v>49</v>
+      </c>
+      <c r="H12" t="s">
+        <v>36</v>
+      </c>
+      <c r="I12">
         <v>24</v>
       </c>
-      <c r="B12" t="s">
-        <v>30</v>
-      </c>
-      <c r="C12">
-        <v>25633</v>
-      </c>
-      <c r="D12" t="s">
-        <v>17</v>
-      </c>
-      <c r="E12" t="s">
-        <v>18</v>
-      </c>
-      <c r="F12">
-        <v>33</v>
-      </c>
-      <c r="G12" t="s">
-        <v>38</v>
-      </c>
-      <c r="H12" t="s">
-        <v>39</v>
-      </c>
-      <c r="I12">
-        <v>10</v>
-      </c>
       <c r="K12" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B13" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C13">
-        <v>32961</v>
+        <v>79135</v>
       </c>
       <c r="D13" t="s">
-        <v>43</v>
+        <v>17</v>
       </c>
       <c r="E13" t="s">
-        <v>45</v>
+        <v>18</v>
       </c>
       <c r="F13">
-        <v>21</v>
+        <v>33</v>
       </c>
       <c r="G13" t="s">
-        <v>58</v>
+        <v>38</v>
       </c>
       <c r="H13" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="I13">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="K13" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B14" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C14">
-        <v>17107</v>
+        <v>18165</v>
       </c>
       <c r="D14" t="s">
-        <v>19</v>
+        <v>43</v>
       </c>
       <c r="E14" t="s">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="F14">
-        <v>44</v>
+        <v>21</v>
       </c>
       <c r="G14" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="H14" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="I14">
-        <v>17</v>
-      </c>
-      <c r="J14" t="s">
-        <v>48</v>
+        <v>5</v>
       </c>
       <c r="K14" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>51</v>
+        <v>26</v>
       </c>
       <c r="B15" t="s">
-        <v>52</v>
+        <v>30</v>
       </c>
       <c r="C15">
-        <v>84963</v>
+        <v>-1</v>
       </c>
       <c r="D15" t="s">
-        <v>53</v>
+        <v>19</v>
       </c>
       <c r="E15" t="s">
-        <v>57</v>
+        <v>20</v>
       </c>
       <c r="F15">
-        <v>21</v>
+        <v>44</v>
       </c>
       <c r="G15" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="H15" t="s">
-        <v>55</v>
+        <v>44</v>
       </c>
       <c r="I15">
-        <v>56</v>
+        <v>17</v>
       </c>
       <c r="J15" t="s">
         <v>48</v>
       </c>
       <c r="K15" t="s">
-        <v>56</v>
+        <v>13</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>51</v>
+      </c>
+      <c r="B16" t="s">
+        <v>52</v>
+      </c>
+      <c r="D16" t="s">
+        <v>53</v>
+      </c>
+      <c r="E16" t="s">
+        <v>57</v>
+      </c>
+      <c r="F16">
         <v>21</v>
       </c>
-      <c r="B16" t="s">
-        <v>28</v>
-      </c>
-      <c r="C16">
-        <v>25641</v>
-      </c>
-      <c r="D16" t="s">
-        <v>41</v>
-      </c>
-      <c r="E16" t="s">
-        <v>1</v>
-      </c>
-      <c r="F16">
-        <v>24</v>
-      </c>
       <c r="G16" t="s">
-        <v>33</v>
+        <v>54</v>
       </c>
       <c r="H16" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="I16">
-        <v>154</v>
+        <v>56</v>
+      </c>
+      <c r="J16" t="s">
+        <v>48</v>
       </c>
       <c r="K16" t="s">
-        <v>8</v>
+        <v>56</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B17" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C17">
-        <v>78945</v>
+        <v>30307</v>
       </c>
       <c r="D17" t="s">
-        <v>14</v>
+        <v>41</v>
       </c>
       <c r="E17" t="s">
-        <v>46</v>
+        <v>1</v>
       </c>
       <c r="F17">
-        <v>55</v>
+        <v>24</v>
       </c>
       <c r="G17" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H17" t="s">
-        <v>35</v>
+        <v>47</v>
       </c>
       <c r="I17">
-        <v>60</v>
-      </c>
-      <c r="J17" t="s">
-        <v>48</v>
+        <v>154</v>
       </c>
       <c r="K17" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B18" t="s">
         <v>27</v>
       </c>
       <c r="C18">
-        <v>25846</v>
+        <v>35454</v>
       </c>
       <c r="D18" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E18" t="s">
-        <v>16</v>
+        <v>46</v>
       </c>
       <c r="F18">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="G18" t="s">
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="H18" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="I18">
-        <v>24</v>
+        <v>60</v>
+      </c>
+      <c r="J18" t="s">
+        <v>48</v>
       </c>
       <c r="K18" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>23</v>
+      </c>
+      <c r="B19" t="s">
+        <v>27</v>
+      </c>
+      <c r="C19">
+        <v>13703</v>
+      </c>
+      <c r="D19" t="s">
+        <v>15</v>
+      </c>
+      <c r="E19" t="s">
+        <v>16</v>
+      </c>
+      <c r="F19">
+        <v>44</v>
+      </c>
+      <c r="G19" t="s">
+        <v>49</v>
+      </c>
+      <c r="H19" t="s">
+        <v>36</v>
+      </c>
+      <c r="I19">
         <v>24</v>
       </c>
-      <c r="B19" t="s">
-        <v>30</v>
-      </c>
-      <c r="C19">
-        <v>79135</v>
-      </c>
-      <c r="D19" t="s">
-        <v>17</v>
-      </c>
-      <c r="E19" t="s">
-        <v>18</v>
-      </c>
-      <c r="F19">
-        <v>33</v>
-      </c>
-      <c r="G19" t="s">
-        <v>38</v>
-      </c>
-      <c r="H19" t="s">
-        <v>39</v>
-      </c>
-      <c r="I19">
-        <v>10</v>
-      </c>
       <c r="K19" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B20" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C20">
-        <v>18165</v>
+        <v>25633</v>
       </c>
       <c r="D20" t="s">
-        <v>43</v>
+        <v>17</v>
       </c>
       <c r="E20" t="s">
-        <v>45</v>
+        <v>18</v>
       </c>
       <c r="F20">
-        <v>21</v>
+        <v>33</v>
       </c>
       <c r="G20" t="s">
-        <v>58</v>
+        <v>38</v>
       </c>
       <c r="H20" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="I20">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="K20" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B21" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C21">
-        <v>-1</v>
+        <v>32961</v>
       </c>
       <c r="D21" t="s">
-        <v>19</v>
+        <v>43</v>
       </c>
       <c r="E21" t="s">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="F21">
-        <v>44</v>
+        <v>21</v>
       </c>
       <c r="G21" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="H21" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="I21">
-        <v>17</v>
-      </c>
-      <c r="J21" t="s">
-        <v>48</v>
+        <v>5</v>
       </c>
       <c r="K21" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>51</v>
+        <v>26</v>
       </c>
       <c r="B22" t="s">
-        <v>52</v>
+        <v>30</v>
+      </c>
+      <c r="C22">
+        <v>17107</v>
       </c>
       <c r="D22" t="s">
-        <v>53</v>
+        <v>19</v>
       </c>
       <c r="E22" t="s">
-        <v>57</v>
+        <v>20</v>
       </c>
       <c r="F22">
-        <v>21</v>
+        <v>44</v>
       </c>
       <c r="G22" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="H22" t="s">
-        <v>55</v>
+        <v>44</v>
       </c>
       <c r="I22">
-        <v>56</v>
+        <v>17</v>
       </c>
       <c r="J22" t="s">
         <v>48</v>
       </c>
       <c r="K22" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>21</v>
-      </c>
-      <c r="B23" t="s">
-        <v>28</v>
-      </c>
-      <c r="C23">
-        <v>30307</v>
-      </c>
-      <c r="D23" t="s">
-        <v>41</v>
-      </c>
-      <c r="E23" t="s">
-        <v>1</v>
-      </c>
-      <c r="F23">
-        <v>24</v>
-      </c>
-      <c r="G23" t="s">
-        <v>33</v>
-      </c>
-      <c r="H23" t="s">
-        <v>47</v>
-      </c>
-      <c r="I23">
-        <v>154</v>
-      </c>
-      <c r="K23" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>22</v>
+        <v>59</v>
       </c>
       <c r="B24" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C24">
-        <v>35454</v>
+        <v>30307</v>
       </c>
       <c r="D24" t="s">
-        <v>14</v>
+        <v>41</v>
       </c>
       <c r="E24" t="s">
-        <v>46</v>
+        <v>1</v>
       </c>
       <c r="F24">
-        <v>55</v>
+        <v>24</v>
       </c>
       <c r="G24" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H24" t="s">
-        <v>35</v>
+        <v>47</v>
       </c>
       <c r="I24">
-        <v>60</v>
-      </c>
-      <c r="J24" t="s">
-        <v>48</v>
+        <v>154</v>
       </c>
       <c r="K24" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B25" t="s">
         <v>27</v>
       </c>
       <c r="C25">
-        <v>13703</v>
+        <v>35454</v>
       </c>
       <c r="D25" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E25" t="s">
-        <v>16</v>
+        <v>46</v>
       </c>
       <c r="F25">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="G25" t="s">
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="H25" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="I25">
-        <v>24</v>
+        <v>60</v>
+      </c>
+      <c r="J25" t="s">
+        <v>48</v>
       </c>
       <c r="K25" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
+        <v>23</v>
+      </c>
+      <c r="B26" t="s">
+        <v>27</v>
+      </c>
+      <c r="C26">
+        <v>13703</v>
+      </c>
+      <c r="D26" t="s">
+        <v>15</v>
+      </c>
+      <c r="E26" t="s">
+        <v>16</v>
+      </c>
+      <c r="F26">
+        <v>44</v>
+      </c>
+      <c r="G26" t="s">
+        <v>49</v>
+      </c>
+      <c r="H26" t="s">
+        <v>36</v>
+      </c>
+      <c r="I26">
         <v>24</v>
       </c>
-      <c r="B26" t="s">
-        <v>30</v>
-      </c>
-      <c r="C26">
-        <v>25633</v>
-      </c>
-      <c r="D26" t="s">
-        <v>17</v>
-      </c>
-      <c r="E26" t="s">
-        <v>18</v>
-      </c>
-      <c r="F26">
-        <v>33</v>
-      </c>
-      <c r="G26" t="s">
-        <v>38</v>
-      </c>
-      <c r="H26" t="s">
-        <v>39</v>
-      </c>
-      <c r="I26">
-        <v>10</v>
-      </c>
       <c r="K26" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B27" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C27">
-        <v>32961</v>
+        <v>25633</v>
       </c>
       <c r="D27" t="s">
-        <v>43</v>
+        <v>17</v>
       </c>
       <c r="E27" t="s">
-        <v>45</v>
+        <v>18</v>
       </c>
       <c r="F27">
-        <v>21</v>
+        <v>33</v>
       </c>
       <c r="G27" t="s">
-        <v>58</v>
+        <v>38</v>
       </c>
       <c r="H27" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="I27">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="K27" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
+        <v>25</v>
+      </c>
+      <c r="B28" t="s">
+        <v>29</v>
+      </c>
+      <c r="C28">
+        <v>32961</v>
+      </c>
+      <c r="D28" t="s">
+        <v>43</v>
+      </c>
+      <c r="E28" t="s">
+        <v>45</v>
+      </c>
+      <c r="F28">
+        <v>21</v>
+      </c>
+      <c r="G28" t="s">
+        <v>58</v>
+      </c>
+      <c r="H28" t="s">
+        <v>40</v>
+      </c>
+      <c r="I28">
+        <v>5</v>
+      </c>
+      <c r="K28" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
         <v>26</v>
       </c>
-      <c r="B28" t="s">
+      <c r="B29" t="s">
         <v>30</v>
       </c>
-      <c r="C28">
+      <c r="C29">
         <v>17107</v>
       </c>
-      <c r="D28" t="s">
+      <c r="D29" t="s">
         <v>19</v>
       </c>
-      <c r="E28" t="s">
+      <c r="E29" t="s">
         <v>20</v>
       </c>
-      <c r="F28">
+      <c r="F29">
         <v>44</v>
       </c>
-      <c r="G28" t="s">
+      <c r="G29" t="s">
         <v>50</v>
       </c>
-      <c r="H28" t="s">
+      <c r="H29" t="s">
         <v>44</v>
       </c>
-      <c r="I28">
+      <c r="I29">
         <v>17</v>
       </c>
-      <c r="J28" t="s">
+      <c r="J29" t="s">
         <v>48</v>
       </c>
-      <c r="K28" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>59</v>
-      </c>
-      <c r="B30" t="s">
-        <v>28</v>
-      </c>
-      <c r="C30">
-        <v>30307</v>
-      </c>
-      <c r="D30" t="s">
-        <v>41</v>
-      </c>
-      <c r="E30" t="s">
-        <v>1</v>
-      </c>
-      <c r="F30">
-        <v>24</v>
-      </c>
-      <c r="G30" t="s">
-        <v>33</v>
-      </c>
-      <c r="H30" t="s">
-        <v>47</v>
-      </c>
-      <c r="I30">
-        <v>154</v>
-      </c>
-      <c r="K30" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>22</v>
-      </c>
-      <c r="B31" t="s">
-        <v>27</v>
-      </c>
-      <c r="C31">
-        <v>35454</v>
-      </c>
-      <c r="D31" t="s">
-        <v>14</v>
-      </c>
-      <c r="E31" t="s">
-        <v>46</v>
-      </c>
-      <c r="F31">
-        <v>55</v>
-      </c>
-      <c r="G31" t="s">
-        <v>34</v>
-      </c>
-      <c r="H31" t="s">
-        <v>35</v>
-      </c>
-      <c r="I31">
-        <v>60</v>
-      </c>
-      <c r="J31" t="s">
-        <v>48</v>
-      </c>
-      <c r="K31" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>23</v>
-      </c>
-      <c r="B32" t="s">
-        <v>27</v>
-      </c>
-      <c r="C32">
-        <v>13703</v>
-      </c>
-      <c r="D32" t="s">
-        <v>15</v>
-      </c>
-      <c r="E32" t="s">
-        <v>16</v>
-      </c>
-      <c r="F32">
-        <v>44</v>
-      </c>
-      <c r="G32" t="s">
-        <v>49</v>
-      </c>
-      <c r="H32" t="s">
-        <v>36</v>
-      </c>
-      <c r="I32">
-        <v>24</v>
-      </c>
-      <c r="K32" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>24</v>
-      </c>
-      <c r="B33" t="s">
-        <v>30</v>
-      </c>
-      <c r="C33">
-        <v>25633</v>
-      </c>
-      <c r="D33" t="s">
-        <v>17</v>
-      </c>
-      <c r="E33" t="s">
-        <v>18</v>
-      </c>
-      <c r="F33">
-        <v>33</v>
-      </c>
-      <c r="G33" t="s">
-        <v>38</v>
-      </c>
-      <c r="H33" t="s">
-        <v>39</v>
-      </c>
-      <c r="I33">
-        <v>10</v>
-      </c>
-      <c r="K33" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>25</v>
-      </c>
-      <c r="B34" t="s">
-        <v>29</v>
-      </c>
-      <c r="C34">
-        <v>32961</v>
-      </c>
-      <c r="D34" t="s">
-        <v>43</v>
-      </c>
-      <c r="E34" t="s">
-        <v>45</v>
-      </c>
-      <c r="F34">
-        <v>21</v>
-      </c>
-      <c r="G34" t="s">
-        <v>58</v>
-      </c>
-      <c r="H34" t="s">
-        <v>40</v>
-      </c>
-      <c r="I34">
-        <v>5</v>
-      </c>
-      <c r="K34" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>26</v>
-      </c>
-      <c r="B35" t="s">
-        <v>30</v>
-      </c>
-      <c r="C35">
-        <v>17107</v>
-      </c>
-      <c r="D35" t="s">
-        <v>19</v>
-      </c>
-      <c r="E35" t="s">
-        <v>20</v>
-      </c>
-      <c r="F35">
-        <v>44</v>
-      </c>
-      <c r="G35" t="s">
-        <v>50</v>
-      </c>
-      <c r="H35" t="s">
-        <v>44</v>
-      </c>
-      <c r="I35">
-        <v>17</v>
-      </c>
-      <c r="J35" t="s">
-        <v>48</v>
-      </c>
-      <c r="K35" t="s">
+      <c r="K29" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1703,6 +1505,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="392a115a-1654-4bb7-9988-dca16703408a" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="88db13ce-348c-49a2-8d98-81b888e52361">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100F14612CBFD8E3740906A56EC3133312A" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b8d8bbe8caf11baa820866fa2f569c06">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="88db13ce-348c-49a2-8d98-81b888e52361" xmlns:ns3="392a115a-1654-4bb7-9988-dca16703408a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="823c8a0d155e31ed95da462af31d249a" ns2:_="" ns3:_="">
     <xsd:import namespace="88db13ce-348c-49a2-8d98-81b888e52361"/>
@@ -1909,27 +1731,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{21854188-CB67-482C-9A8D-10A223339233}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="88db13ce-348c-49a2-8d98-81b888e52361"/>
+    <ds:schemaRef ds:uri="392a115a-1654-4bb7-9988-dca16703408a"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="392a115a-1654-4bb7-9988-dca16703408a" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="88db13ce-348c-49a2-8d98-81b888e52361">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{952BBB55-DF49-49C2-B3DD-6A3C0584915B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C11CCDF0-8CE4-48A7-8939-80C6ED574B29}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1946,29 +1773,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{952BBB55-DF49-49C2-B3DD-6A3C0584915B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{21854188-CB67-482C-9A8D-10A223339233}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="88db13ce-348c-49a2-8d98-81b888e52361"/>
-    <ds:schemaRef ds:uri="392a115a-1654-4bb7-9988-dca16703408a"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>